<commit_message>
Added new RDF data schemes and visual schemes for employment-table09-10, fixed XLSX spreadsheet for employment-table10
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table10.xlsx
+++ b/sources/table_normalization/xlsx/employment-table10.xlsx
@@ -115,7 +115,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -134,6 +134,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -147,15 +153,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -462,18 +469,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -481,18 +488,18 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
+      <c r="E4" s="2"/>
+      <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="5"/>
@@ -521,7 +528,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B8">
@@ -544,7 +551,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B9">
@@ -894,7 +901,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="A26" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B26">
@@ -917,7 +924,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="A27" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B27">
@@ -1267,7 +1274,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="A44" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B44">
@@ -1290,7 +1297,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="A45" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B45">
@@ -1640,7 +1647,7 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+      <c r="A62" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B62">
@@ -1663,7 +1670,7 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+      <c r="A63" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B63">
@@ -2013,7 +2020,7 @@
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+      <c r="A80" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B80">
@@ -2036,7 +2043,7 @@
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+      <c r="A81" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B81">
@@ -2381,15 +2388,15 @@
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A97" s="2" t="s">
+      <c r="A97" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="2"/>
-      <c r="G97" s="2"/>
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+      <c r="F97" s="4"/>
+      <c r="G97" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>